<commit_message>
Agregado modulo geografico por departamentos y analisis por trimestre y ano de nacimiento
</commit_message>
<xml_diff>
--- a/DATOS INDIVIDUALES.xlsx
+++ b/DATOS INDIVIDUALES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Desktop/Dashboard_Fortaleza/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/Dashboard Forta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{856A172B-AEB3-9C46-9D72-2936651CD7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD12A071-0F19-6643-8AF3-39BA79AB108F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3253,6 +3253,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:79" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Lectura directa desde Resumen_Jugadores para corregir mes y trimestre
</commit_message>
<xml_diff>
--- a/DATOS INDIVIDUALES.xlsx
+++ b/DATOS INDIVIDUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/Dashboard Forta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD12A071-0F19-6643-8AF3-39BA79AB108F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D034416-441E-814F-AD16-2CE3F78FF8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen_Jugadores" sheetId="1" r:id="rId1"/>
@@ -859,6 +859,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.5" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">

</xml_diff>